<commit_message>
Kd-Conversion.xlsx now contains r^2 values.
</commit_message>
<xml_diff>
--- a/KD-Conversion.xlsx
+++ b/KD-Conversion.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uncw4-my.sharepoint.com/personal/dem5075_uncw_edu/Documents/SSD/src/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uncw4-my.sharepoint.com/personal/dem5075_uncw_edu/Documents/SSD/Sensing-Secchi-Disk-COAST/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1" documentId="11_457922FD2ABC6DFCA567243282380D5714411EB3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0187A6C2-1F03-FE46-8495-18A9A8620DB1}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="620" windowWidth="38400" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kd" sheetId="1" r:id="rId1"/>

</xml_diff>